<commit_message>
Added letter of intent
Letter of Intent to apply for tenure and promotion
</commit_message>
<xml_diff>
--- a/2_Teaching_Effectiveness/2b_Student_Course_Evaluations/Z_Misc/Course Evaluation Numbers.xlsx
+++ b/2_Teaching_Effectiveness/2b_Student_Course_Evaluations/Z_Misc/Course Evaluation Numbers.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dcham\Documents\GitHub\Chamberlain_Tenure_Packet\2_Teaching_Effectiveness\2b_Student_Course_Evaluations\Z_Misc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F7C5ADA-6A4D-4325-9ABD-53B2DEA15D50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A26EF7E-591A-4ABB-831C-E9A1C4041565}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1305" yWindow="2430" windowWidth="16755" windowHeight="17655" xr2:uid="{2882075C-5BCF-BB48-99E2-FB2C0697CBA8}"/>
+    <workbookView xWindow="8475" yWindow="1920" windowWidth="17505" windowHeight="17655" xr2:uid="{2882075C-5BCF-BB48-99E2-FB2C0697CBA8}"/>
   </bookViews>
   <sheets>
     <sheet name="metrics" sheetId="1" r:id="rId1"/>
@@ -232,7 +232,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -257,6 +257,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1643,8 +1644,27 @@
       <c r="D38">
         <v>9</v>
       </c>
-      <c r="H38" s="6"/>
-      <c r="K38" s="6"/>
+      <c r="E38">
+        <v>6</v>
+      </c>
+      <c r="F38">
+        <v>5</v>
+      </c>
+      <c r="G38">
+        <v>4.6500000000000004</v>
+      </c>
+      <c r="H38" s="6">
+        <v>4.62</v>
+      </c>
+      <c r="I38" s="18">
+        <v>3</v>
+      </c>
+      <c r="J38" s="18">
+        <v>0</v>
+      </c>
+      <c r="K38" s="6">
+        <v>0</v>
+      </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" s="5" t="s">
@@ -1660,8 +1680,27 @@
       <c r="D39">
         <v>25</v>
       </c>
-      <c r="H39" s="6"/>
-      <c r="K39" s="6"/>
+      <c r="E39">
+        <v>17</v>
+      </c>
+      <c r="F39">
+        <v>4.71</v>
+      </c>
+      <c r="G39">
+        <v>4.6500000000000004</v>
+      </c>
+      <c r="H39" s="6">
+        <v>4.62</v>
+      </c>
+      <c r="I39" s="18">
+        <v>1</v>
+      </c>
+      <c r="J39" s="18">
+        <v>0</v>
+      </c>
+      <c r="K39" s="6">
+        <v>0</v>
+      </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" s="5" t="s">
@@ -1710,11 +1749,11 @@
       </c>
       <c r="E42">
         <f>SUM(E2:E41)</f>
-        <v>245</v>
+        <v>268</v>
       </c>
       <c r="F42" s="17">
         <f>SUMPRODUCT(E2:E41,F2:F41)/E42</f>
-        <v>4.6589387755102036</v>
+        <v>4.6698134328358201</v>
       </c>
       <c r="G42" s="13" t="s">
         <v>24</v>
@@ -1724,7 +1763,7 @@
       </c>
       <c r="I42">
         <f>SUM(I2:I41)</f>
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="J42">
         <f>SUM(J2:J41)</f>

</xml_diff>